<commit_message>
edit to filinia without width
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Erie/D20/Rots/ER 59 D20 Spring 2024 24GE03I14 Rot.xlsx
+++ b/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Erie/D20/Rots/ER 59 D20 Spring 2024 24GE03I14 Rot.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccm243\OneDrive - Cornell University\Desktop\GLNPO Counts\2024\Spring\Erie\d20\Rot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\GLNPO 2024 Spring\Erie\D20\Rots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48E304F-2B4B-4FB6-82EF-2C4F14E06EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1E78C3-F5D4-4233-9AE5-7D450E509900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C8B736CF-5FB0-44B6-968D-4BEC76E90384}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C8B736CF-5FB0-44B6-968D-4BEC76E90384}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2261" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -379,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -387,7 +387,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2344,7 +2343,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C326082C-6289-4CDD-98C4-A0BCB9CF8AA0}" name="PivotTable3" cacheId="2261" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C326082C-6289-4CDD-98C4-A0BCB9CF8AA0}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="X4:AA15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField showAll="0"/>
@@ -2771,19 +2770,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595CA4D2-4C24-43E3-BBB0-4A9DF4F915D5}">
   <dimension ref="A1:AA77"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.7265625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.1796875" customWidth="1"/>
-    <col min="27" max="27" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.21875" customWidth="1"/>
+    <col min="27" max="27" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2851,7 +2850,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -2910,7 +2909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -2969,7 +2968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -3034,7 +3033,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -3105,7 +3104,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -3166,15 +3165,14 @@
       <c r="X6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="Y6" s="5">
-        <v>1</v>
-      </c>
-      <c r="Z6" s="5"/>
-      <c r="AA6" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="AA6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -3235,15 +3233,14 @@
       <c r="X7" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="Y7" s="5">
+      <c r="Y7">
         <v>2</v>
       </c>
-      <c r="Z7" s="5"/>
-      <c r="AA7" s="5">
+      <c r="AA7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -3304,17 +3301,17 @@
       <c r="X8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="Y8" s="5">
+      <c r="Y8">
         <v>97</v>
       </c>
-      <c r="Z8" s="5">
+      <c r="Z8">
         <v>125</v>
       </c>
-      <c r="AA8" s="5">
+      <c r="AA8">
         <v>222</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -3375,17 +3372,17 @@
       <c r="X9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="Y9" s="5">
+      <c r="Y9">
         <v>465</v>
       </c>
-      <c r="Z9" s="5">
+      <c r="Z9">
         <v>445</v>
       </c>
-      <c r="AA9" s="5">
+      <c r="AA9">
         <v>910</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3446,15 +3443,14 @@
       <c r="X10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="Y10" s="5"/>
-      <c r="Z10" s="5">
-        <v>1</v>
-      </c>
-      <c r="AA10" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -3515,15 +3511,14 @@
       <c r="X11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="Y11" s="5"/>
-      <c r="Z11" s="5">
+      <c r="Z11">
         <v>2</v>
       </c>
-      <c r="AA11" s="5">
+      <c r="AA11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -3584,15 +3579,14 @@
       <c r="X12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="Y12" s="5">
-        <v>1</v>
-      </c>
-      <c r="Z12" s="5"/>
-      <c r="AA12" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="Y12">
+        <v>1</v>
+      </c>
+      <c r="AA12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -3653,15 +3647,14 @@
       <c r="X13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Y13" s="5">
+      <c r="Y13">
         <v>3</v>
       </c>
-      <c r="Z13" s="5"/>
-      <c r="AA13" s="5">
+      <c r="AA13">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -3722,17 +3715,17 @@
       <c r="X14" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="Y14" s="5">
+      <c r="Y14">
         <v>69</v>
       </c>
-      <c r="Z14" s="5">
+      <c r="Z14">
         <v>73</v>
       </c>
-      <c r="AA14" s="5">
+      <c r="AA14">
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -3793,17 +3786,17 @@
       <c r="X15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="Y15" s="5">
+      <c r="Y15">
         <v>638</v>
       </c>
-      <c r="Z15" s="5">
+      <c r="Z15">
         <v>646</v>
       </c>
-      <c r="AA15" s="5">
+      <c r="AA15">
         <v>1284</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -3862,7 +3855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -3921,7 +3914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -3979,17 +3972,17 @@
       <c r="U18">
         <v>1</v>
       </c>
-      <c r="X18" s="6" t="s">
+      <c r="X18" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="Y18" s="7" t="s">
+      <c r="Y18" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="Z18" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+      <c r="Z18" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -4047,15 +4040,15 @@
       <c r="U19">
         <v>1</v>
       </c>
-      <c r="X19" s="9"/>
-      <c r="Y19" s="7" t="s">
+      <c r="X19" s="8"/>
+      <c r="Y19" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="Z19" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+      <c r="Z19" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -4113,17 +4106,17 @@
       <c r="U20">
         <v>1</v>
       </c>
-      <c r="X20" s="6" t="s">
+      <c r="X20" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="Y20" s="7" t="s">
+      <c r="Y20" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="Z20" s="8">
+      <c r="Z20" s="7">
         <v>1.0009999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -4181,15 +4174,15 @@
       <c r="U21">
         <v>1</v>
       </c>
-      <c r="X21" s="9"/>
-      <c r="Y21" s="7" t="s">
+      <c r="X21" s="8"/>
+      <c r="Y21" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="Z21" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+      <c r="Z21" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -4247,15 +4240,15 @@
       <c r="U22">
         <v>1</v>
       </c>
-      <c r="X22" s="10" t="s">
+      <c r="X22" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="Y22" s="11" t="s">
+      <c r="Y22" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="Z22" s="12"/>
-    </row>
-    <row r="23" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+      <c r="Z22" s="11"/>
+    </row>
+    <row r="23" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -4313,15 +4306,15 @@
       <c r="U23">
         <v>1</v>
       </c>
-      <c r="X23" s="10" t="s">
+      <c r="X23" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Y23" s="11" t="s">
+      <c r="Y23" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="Z23" s="12"/>
-    </row>
-    <row r="24" spans="1:26" ht="16" x14ac:dyDescent="0.4">
+      <c r="Z23" s="11"/>
+    </row>
+    <row r="24" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -4379,13 +4372,13 @@
       <c r="U24">
         <v>1</v>
       </c>
-      <c r="X24" s="7" t="s">
+      <c r="X24" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="Y24" s="11"/>
-      <c r="Z24" s="12"/>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="Y24" s="10"/>
+      <c r="Z24" s="11"/>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -4444,7 +4437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>22</v>
       </c>
@@ -4503,7 +4496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -4562,7 +4555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -4621,7 +4614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -4680,7 +4673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -4739,7 +4732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>22</v>
       </c>
@@ -4798,7 +4791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -4857,7 +4850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -4916,7 +4909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -4975,7 +4968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>22</v>
       </c>
@@ -5034,7 +5027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>22</v>
       </c>
@@ -5093,7 +5086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -5152,7 +5145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -5211,7 +5204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>22</v>
       </c>
@@ -5270,7 +5263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>22</v>
       </c>
@@ -5329,7 +5322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>22</v>
       </c>
@@ -5388,7 +5381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -5447,7 +5440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>22</v>
       </c>
@@ -5506,7 +5499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -5565,7 +5558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -5624,7 +5617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -5683,7 +5676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>22</v>
       </c>
@@ -5742,7 +5735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>22</v>
       </c>
@@ -5801,7 +5794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>22</v>
       </c>
@@ -5860,7 +5853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>22</v>
       </c>
@@ -5919,7 +5912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>22</v>
       </c>
@@ -5978,7 +5971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>22</v>
       </c>
@@ -6037,7 +6030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>22</v>
       </c>
@@ -6096,7 +6089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>22</v>
       </c>
@@ -6155,7 +6148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>22</v>
       </c>
@@ -6214,7 +6207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>22</v>
       </c>
@@ -6273,7 +6266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -6332,7 +6325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>22</v>
       </c>
@@ -6391,7 +6384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>22</v>
       </c>
@@ -6450,7 +6443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>22</v>
       </c>
@@ -6509,7 +6502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>22</v>
       </c>
@@ -6568,7 +6561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>22</v>
       </c>
@@ -6627,7 +6620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>22</v>
       </c>
@@ -6686,7 +6679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>22</v>
       </c>
@@ -6745,7 +6738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>22</v>
       </c>
@@ -6804,7 +6797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>22</v>
       </c>
@@ -6863,7 +6856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>22</v>
       </c>
@@ -6922,7 +6915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -6981,7 +6974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>22</v>
       </c>
@@ -7040,7 +7033,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>22</v>
       </c>
@@ -7099,7 +7092,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>22</v>
       </c>
@@ -7158,7 +7151,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>22</v>
       </c>
@@ -7211,13 +7204,13 @@
         <v>0.18</v>
       </c>
       <c r="T72">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="U72">
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>22</v>
       </c>
@@ -7276,7 +7269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>22</v>
       </c>
@@ -7335,7 +7328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>22</v>
       </c>
@@ -7394,7 +7387,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>22</v>
       </c>
@@ -7453,7 +7446,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>22</v>
       </c>

</xml_diff>